<commit_message>
migrate(5-3): bundle & component optimizations
</commit_message>
<xml_diff>
--- a/docs/migration-orders/prompt-to-claude-code/antigravity/migration-process-handbook-antigravity-v4.xlsx
+++ b/docs/migration-orders/prompt-to-claude-code/antigravity/migration-process-handbook-antigravity-v4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SaaS Project\trading-alerts-saas-public\docs\migration-orders\prompt-to-claude-code\antigravity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{165368FB-9F91-48DB-83DA-B87E6CB0A8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61BE81F3-5A01-43D4-B1E4-E59EC5D5A559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Audit_Report" sheetId="1" r:id="rId1"/>
@@ -3588,7 +3588,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -3738,6 +3738,18 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10446,22 +10458,22 @@
       </c>
     </row>
     <row r="59" spans="1:18" ht="158.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A59" s="2">
+      <c r="A59" s="68">
         <v>58</v>
       </c>
-      <c r="B59" s="14" t="s">
+      <c r="B59" s="60" t="s">
         <v>463</v>
       </c>
-      <c r="C59" s="15" t="s">
+      <c r="C59" s="69" t="s">
         <v>464</v>
       </c>
-      <c r="D59" s="3" t="s">
+      <c r="D59" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="E59" s="16" t="s">
+      <c r="E59" s="70" t="s">
         <v>853</v>
       </c>
-      <c r="F59" s="16" t="s">
+      <c r="F59" s="70" t="s">
         <v>854</v>
       </c>
       <c r="G59" s="16" t="s">
@@ -10502,20 +10514,20 @@
       </c>
     </row>
     <row r="60" spans="1:18" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A60" s="2">
+      <c r="A60" s="68">
         <v>59</v>
       </c>
-      <c r="B60" s="14" t="s">
+      <c r="B60" s="60" t="s">
         <v>470</v>
       </c>
-      <c r="C60" s="15" t="s">
+      <c r="C60" s="69" t="s">
         <v>464</v>
       </c>
-      <c r="D60" s="3" t="s">
+      <c r="D60" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="E60" s="13"/>
-      <c r="F60" s="16" t="s">
+      <c r="E60" s="71"/>
+      <c r="F60" s="70" t="s">
         <v>859</v>
       </c>
       <c r="G60" s="16" t="s">
@@ -10552,20 +10564,20 @@
       </c>
     </row>
     <row r="61" spans="1:18" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A61" s="2">
+      <c r="A61" s="68">
         <v>60</v>
       </c>
-      <c r="B61" s="14" t="s">
+      <c r="B61" s="60" t="s">
         <v>476</v>
       </c>
-      <c r="C61" s="15" t="s">
+      <c r="C61" s="69" t="s">
         <v>464</v>
       </c>
-      <c r="D61" s="3" t="s">
+      <c r="D61" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="E61" s="13"/>
-      <c r="F61" s="16" t="s">
+      <c r="E61" s="71"/>
+      <c r="F61" s="70" t="s">
         <v>863</v>
       </c>
       <c r="G61" s="16" t="s">
@@ -10602,20 +10614,20 @@
       </c>
     </row>
     <row r="62" spans="1:18" ht="172.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A62" s="2">
+      <c r="A62" s="68">
         <v>61</v>
       </c>
-      <c r="B62" s="14" t="s">
+      <c r="B62" s="60" t="s">
         <v>481</v>
       </c>
-      <c r="C62" s="15" t="s">
+      <c r="C62" s="69" t="s">
         <v>464</v>
       </c>
-      <c r="D62" s="3" t="s">
+      <c r="D62" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="E62" s="13"/>
-      <c r="F62" s="16" t="s">
+      <c r="E62" s="71"/>
+      <c r="F62" s="70" t="s">
         <v>867</v>
       </c>
       <c r="G62" s="16" t="s">

</xml_diff>